<commit_message>
Add Gateway SP invoice status tab to SR status reference workbook
New tab 'SP Invoice Status (Gateway)' with invoice.status values from
Gateway AP skills. Includes build script that samples live Gateway MCP
when GATEWAY_API_TOKEN is configured.

Co-authored-by: Crystal Gagner <crysgagner@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/vixxo-sr-status-reference.xlsx
+++ b/exports/vixxo-sr-status-reference.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="SR Status" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SR Sub-Status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SP Invoice Status (Gateway)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +53,11 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -74,6 +80,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +470,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -882,7 +888,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1859,7 +1864,6 @@
           <t>VixxoLink / Gateway</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>Recently opened/transferred; not yet a health signal</t>
@@ -1887,7 +1891,6 @@
           <t>VixxoLink / Gateway</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>Normal healthy path</t>
@@ -1915,7 +1918,6 @@
           <t>VixxoLink / Gateway</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Borderline; watch closely</t>
@@ -1943,7 +1945,6 @@
           <t>VixxoLink / Gateway</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>Real problem path</t>
@@ -1971,7 +1972,6 @@
           <t>VixxoLink / Gateway</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Positive closed-out condition</t>
@@ -1999,7 +1999,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>Invoice accepted in billing workflow</t>
@@ -2027,7 +2026,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>Invoice billed</t>
@@ -2055,7 +2053,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>Invoice paid</t>
@@ -2083,7 +2080,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>AR investigation hold</t>
@@ -2111,7 +2107,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>AP review required</t>
@@ -2139,7 +2134,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>Visual audit review</t>
@@ -2167,7 +2161,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>Paid-only pending state</t>
@@ -2195,7 +2188,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>Invoice creation pending</t>
@@ -2223,7 +2215,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>Rejected; do not process</t>
@@ -2251,7 +2242,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>Payment disposition label in AP reply drafting</t>
@@ -2279,7 +2269,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>Payment disposition label in AP reply drafting</t>
@@ -2307,7 +2296,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>Payment disposition label in AP reply drafting</t>
@@ -2335,7 +2323,6 @@
           <t>Gateway</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Payment disposition label in AP reply drafting</t>
@@ -2354,4 +2341,565 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gateway SP invoice status reference — compiled 2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: workspace-documented Gateway invoice.status values only. Gateway MCP bearer token was not available in this environment — re-run with GATEWAY_API_TOKEN or ~/.vixxo/gateway_api_token to refresh from live Gateway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Invoice Status</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Gateway Field</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Meaning / AP Notes</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Source Reference</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Sample SR</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Sample SP</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Data Origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Creation Pending</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Invoice creation pending in billing system</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Review</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Invoice in AP line-item review (also appears as SR Substatus)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; sub-status-decoder.md</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>PaidOnlyPending</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Paid-only pending state</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>ReviewByAP</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Accounts payable review required</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>UnderARInvestigation</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>AR investigation hold</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>VisualAudit</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>AP review / hold</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Visual audit review</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Delinquent SC Invoice</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Delinquent / vendor billing</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SP missed Service Channel invoice SLA (also SR Substatus)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; sub-status-decoder.md</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Payment lifecycle</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Invoice accepted in billing workflow</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Billed</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Payment lifecycle</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Invoice billed to customer/AP</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Payment lifecycle</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Invoice paid</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>RejectedDoNotProcess</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Rejection</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Rejected; do not process payment</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>vixxo-freshdesk-invoice-review/SKILL.md; starbucks-completed-sr-report/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>AR Successful</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>SR billing overlap</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>AR booked invoice successfully (SR Substatus)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>sub-status-decoder.md</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Required for SR</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>SR billing overlap</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Work complete; SP invoice not yet uploaded (SR Substatus in VixxoLink)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>sub-status-decoder.md; vixxo-spm-invoice-concerns/SKILL.md</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>No Invoice Pending</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>invoice.status</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>SR billing overlap</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>No invoice expected on SR</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>sub-status-decoder.md</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Harden SR status build script for Gateway live picklist refresh
Prefer gateway_list_invoice_statuses when a Gateway OAuth bearer is
available, fall back to gateway_search_invoices sampling, and emit
clear diagnostics when live MCP auth is missing.

Co-authored-by: Crystal Gagner <crysgagner@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/vixxo-sr-status-reference.xlsx
+++ b/exports/vixxo-sr-status-reference.xlsx
@@ -36,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -81,6 +86,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,7 +465,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vixxo SR Status reference — compiled 2026-07-02</t>
+          <t>Vixxo SR Status reference — compiled 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -877,7 +883,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vixxo SR Sub-Status &amp; Invoice Status reference — compiled 2026-07-02</t>
+          <t>Vixxo SR Sub-Status &amp; Invoice Status reference — compiled 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2365,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="59" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2369,10 +2375,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: workspace-documented Gateway invoice.status values only. Gateway MCP bearer token was not available in this environment — re-run with GATEWAY_API_TOKEN or ~/.vixxo/gateway_api_token to refresh from live Gateway.</t>
+          <t>Source: workspace-documented Gateway invoice.status values only. Live Gateway MCP calls failed — picklist: no Gateway bearer token; sample: no Gateway bearer token. Authenticate Gateway MCP in Cursor (OAuth) or set GATEWAY_API_TOKEN / ~/.vixxo/gateway_api_token, then re-run this script.</t>
         </is>
       </c>
     </row>
@@ -2420,478 +2426,478 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Invoice Creation Pending</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Invoice creation pending in billing system</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Invoice Review</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Invoice in AP line-item review (also appears as SR Substatus)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; sub-status-decoder.md</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>PaidOnlyPending</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Paid-only pending state</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>ReviewByAP</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Accounts payable review required</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>UnderARInvestigation</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>AR investigation hold</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>VisualAudit</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>AP review / hold</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Visual audit review</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Delinquent SC Invoice</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Delinquent / vendor billing</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>SP missed Service Channel invoice SLA (also SR Substatus)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; sub-status-decoder.md</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Payment lifecycle</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Invoice accepted in billing workflow</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Billed</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Payment lifecycle</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Invoice billed to customer/AP</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Payment lifecycle</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Invoice paid</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>RejectedDoNotProcess</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Rejection</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Rejected; do not process payment</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>vixxo-freshdesk-invoice-review/SKILL.md; starbucks-completed-sr-report/SKILL.md</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>AR Successful</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>SR billing overlap</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>AR booked invoice successfully (SR Substatus)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>sub-status-decoder.md</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Invoice Required for SR</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>SR billing overlap</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Work complete; SP invoice not yet uploaded (SR Substatus in VixxoLink)</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>sub-status-decoder.md; vixxo-spm-invoice-concerns/SKILL.md</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>No Invoice Pending</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>invoice.status</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>SR billing overlap</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>No invoice expected on SR</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>sub-status-decoder.md</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Workspace documented (Gateway not queried or value not in sample)</t>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Workspace documented (not returned by live Gateway query)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Gateway MCP OAuth connection without API token
Switch Vixxo HTTP MCPs in mcp.json to Cursor url OAuth (gateway,
vixxolink, vixxonow, etc.) instead of npx mcp-remote without auth.
Add mcp_oauth.py to read cached tokens from ~/.mcp-auth for skill scripts,
fast-fail when OAuth is missing, and update diagnose/build tooling.

Co-authored-by: Crystal Gagner <crysgagner@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/vixxo-sr-status-reference.xlsx
+++ b/exports/vixxo-sr-status-reference.xlsx
@@ -36,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -76,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,6 +92,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2378,7 +2384,7 @@
     <row r="2" ht="55" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: workspace-documented Gateway invoice.status values only. Live Gateway MCP calls failed — picklist: no Gateway bearer token; sample: no Gateway bearer token. Authenticate Gateway MCP in Cursor (OAuth) or set GATEWAY_API_TOKEN / ~/.vixxo/gateway_api_token, then re-run this script.</t>
+          <t>Source: workspace-documented Gateway invoice.status values only. Live Gateway MCP calls failed — picklist: gateway_list_invoice_statuses: Gateway/Vixxo MCP OAuth not configured. Connect gateway in Cursor Settings → MCP (url OAuth, no API token), then retry.; sample: gateway_search_invoices returned no invoice rows. Authenticate Gateway MCP in Cursor (Settings → MCP → gateway; OAuth, no API token) or set GATEWAY_API_TOKEN / ~/.vixxo/gateway_api_token, then re-run this script.</t>
         </is>
       </c>
     </row>

</xml_diff>